<commit_message>
worktime excel file python -1h
</commit_message>
<xml_diff>
--- a/Dokumentation/Michael_worktime.xlsx
+++ b/Dokumentation/Michael_worktime.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micha\Documents\Messung_von_Quanteneffecten_in_MOSFETs\Diplom_Arbeit\Dokumentation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Michael Watzek\Documents\Diplom_Arbeit\Dokumentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88C52D36-5222-48C3-96D9-241724387A16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Begleitprotokoll" sheetId="1" r:id="rId1"/>
@@ -7204,6 +7204,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x0101008067AD2B056D8444940990D952018BC3" ma:contentTypeVersion="3" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="93685f8dc5a4bf59adc50d863541630c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d547fa0d-83bc-4f36-8e52-df9a97b34ceb" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5c90d005da77fb96be18ab65d73ee448" ns2:_="">
     <xsd:import namespace="d547fa0d-83bc-4f36-8e52-df9a97b34ceb"/>
@@ -7341,12 +7347,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -7357,6 +7357,22 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D4E0995F-5523-464E-96ED-BF1A4901DFD3}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="7adf83ab-5e43-45ba-a22e-7b0fb05f9f24"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{06EBFCBE-A719-409F-8BE7-AA1A8F7F26CF}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -7374,22 +7390,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D4E0995F-5523-464E-96ED-BF1A4901DFD3}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="7adf83ab-5e43-45ba-a22e-7b0fb05f9f24"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0D4D141D-07A0-4E53-A884-D40FAAA8E67D}">
   <ds:schemaRefs>

</xml_diff>